<commit_message>
feat: replace PUK with card expiry date
Co-authored-by: Copilot App <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/data/customer_cards.xlsx
+++ b/data/customer_cards.xlsx
@@ -461,7 +461,7 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>puk</t>
+          <t>expiry_date</t>
         </is>
       </c>
     </row>
@@ -498,7 +498,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>73918426</t>
+          <t>12/2028</t>
         </is>
       </c>
     </row>
@@ -535,7 +535,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>28461735</t>
+          <t>06/2027</t>
         </is>
       </c>
     </row>
@@ -572,7 +572,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>81642957</t>
+          <t>03/2029</t>
         </is>
       </c>
     </row>
@@ -609,7 +609,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>54219863</t>
+          <t>11/2026</t>
         </is>
       </c>
     </row>

</xml_diff>